<commit_message>
new.py: Added a function to calculate the square of a number
</commit_message>
<xml_diff>
--- a/questions_answers.xlsx
+++ b/questions_answers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\chataddb\stubot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D42F8DB-D7A0-400F-A79C-5C1CD7FB5984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBCB3D5-6FE5-41CA-A9AA-8F07101BFB80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1DAF3C1D-9B04-428E-B9FE-47A514BA530F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>question</t>
   </si>
@@ -169,6 +169,60 @@
   </si>
   <si>
     <t>What is the passing number in  the examination?</t>
+  </si>
+  <si>
+    <t>What kind of support does Anudip offer after I get placed?</t>
+  </si>
+  <si>
+    <t>Anudip offers post-placement follow-ups, guidance for workplace adaptation, and alumni networking opportunities</t>
+  </si>
+  <si>
+    <t>Does Anudip offer any courses in regional languages like Bengali or Hindi?</t>
+  </si>
+  <si>
+    <t>Yes, basic instructions and mentoring are available in regional languages, but digital and soft skill modules are predominantly in English to build employability.</t>
+  </si>
+  <si>
+    <t>I am a person with a disability. Does Anudip have support for me?</t>
+  </si>
+  <si>
+    <t>Yes, Anudip is an inclusive organization. Please contact the Centre Faculty to enquire if there are relevant courses operational for PWD youths.</t>
+  </si>
+  <si>
+    <t>What if I face technical issues logging into online sessions?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please contact the faculty for guidance </t>
+  </si>
+  <si>
+    <t>Will I receive a certificate after completing the course?</t>
+  </si>
+  <si>
+    <t>Yes, a certificate is issued after successful course completion and internal assessment, usually within 15–30 working days. You are encouraged to collect it from your training centre</t>
+  </si>
+  <si>
+    <t>How does Anudip ensure job placements are genuine and safe?</t>
+  </si>
+  <si>
+    <t>All placement partners are verified through a due diligence process, and job offers are tracked for compliance, salary standards, and safety.</t>
+  </si>
+  <si>
+    <t>Can I refer a friend or sibling to enroll in Anudip’s courses?</t>
+  </si>
+  <si>
+    <t>Yes, referrals are welcome. Your friend can apply by walking in to his/her nearest Anudip training centre</t>
+  </si>
+  <si>
+    <t>How can I become part of the Anudip Alumni Network?</t>
+  </si>
+  <si>
+    <t>All placed candidates are encouraged to join Anudip Alumni Network in social media. Please reach out to your faculty for guidance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What if my concern is not listed here ? </t>
+  </si>
+  <si>
+    <t>If your concern is not listed please contact your faculty for any concern/support/guidance</t>
   </si>
 </sst>
 </file>
@@ -521,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6DEF95E-08A4-4BEB-913A-99C70BCF58D5}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="113.1796875" bestFit="1" customWidth="1"/>
@@ -675,58 +729,130 @@
       </c>
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>